<commit_message>
Remove surgical video synthesis entries
</commit_message>
<xml_diff>
--- a/miccai2024.xlsx
+++ b/miccai2024.xlsx
@@ -334,7 +334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -412,35 +412,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>VISAGE: Video Synthesis Using Action Graphs for Surgery (MICCAI 2024 Workshops)</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Laparoscopic surgical video synthesis</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Action graph-guided diffusion video synthesis</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1007/978-3-031-77610-6_14</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Surgical Video Generation</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>